<commit_message>
Format Common_Issues_Sheet.xlsx with professional styling, borders, alternating colors, and auto-filter
Agent-Logs-Url: https://github.com/AhmedAsrar/test/sessions/57e16c19-917b-4c81-9dbc-f7a659de55a9

Co-authored-by: AhmedAsrar <262067190+AhmedAsrar@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Common_Issues_Sheet.xlsx
+++ b/Common_Issues_Sheet.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Common Issues" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Common Issues'!$A$1:$C$72</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +27,44 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+        <bgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +72,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,87 +460,92 @@
   </sheetPr>
   <dimension ref="A1:C72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Common Issue Category</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Reported By</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Original Issue</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>JSON Parse error on Explore/Building page</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>JSON Parse error comes up when user navigates to the building page for the second time from somewhere else.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>JSON Parse error on Explore/Building page</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>In Explore Menu, Building works on very 1st time. If you click back button and retrun to Explore Building again, it returns JSON PARSE Error</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>JSON Parse error on Explore/Building page</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Nihal Mascarenhas</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>error message popping when opening - explore building</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Comfort Management - No rooms / not rendering</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
         <is>
           <t>Inconsistent behaviour between List View and Grid view in Comfort tab as executive.
 List view says "No Rooms" but grid view just shows an empty page without any message.</t>
@@ -503,357 +553,357 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Comfort Management - No rooms / not rendering</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t>In Comfort Management, In List View If no rooms assigned "No rooms found" text there.While in the Grid view it's not there.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Comfort Management - No rooms / not rendering</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Shaharyar Haider</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t>No Rooms found in Monitor -&gt; Comfort</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Comfort Management - No rooms / not rendering</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Comfort page should say that there is no information to be viewed on the page instead of blank page</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Comfort Management - No rooms / not rendering</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Nihal Mascarenhas</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t>Comfot management not rendering</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Font size too small</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Font Size is too small inside the Chart</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Font size too small</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Font Size is too small in this value text</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Font size too small</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Energy Breakdown graph text is too small</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Font size too small</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Text is a little too small</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Icon misalignment in side menu/drawer</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>The Side Menu icons are appearing too close to the labels and the alignment is also not consistent throughout the options</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Icon misalignment in side menu/drawer</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Icons are not aligned</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Icon misalignment in side menu/drawer</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>Nihal Mascarenhas</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Misalignment with other icons in the drawer</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Icon misalignment in side menu/drawer</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr">
         <is>
           <t>Nihal Mascarenhas</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
         <is>
           <t>Top 3 icons and bottom 4 icons are mis aligned</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Back button not working / inconsistent</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>If user goes from "Intellegence &gt; AI Compliance" to "AI Operations &gt; Maintainance" and then press back button, it will take user to the previous page but the same back button behaviour is not consistant throughout the website (e,g, From "Start/Stop" you can't come back to previous page).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Back button not working / inconsistent</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
         <is>
           <t>Back button doesn’t go back to marina plaza, takes me to the same page</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Back button not working / inconsistent</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Back Button should be in same format as other pages</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Back button not working / inconsistent</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Nihal Mascarenhas</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>back bottom does not redirect to anywhere; if user starts on that page</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Back button not working / inconsistent</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="2" t="inlineStr">
         <is>
           <t>Siji Wilson</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Back button is not working in AI report</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Dark mode visibility issues</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="3" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="3" t="inlineStr">
         <is>
           <t>The text in the footer of chat box is not visible in dark mode</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Dark mode visibility issues</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Dark purple font in dark mode is not very reading-friendly</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Dark mode visibility issues</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Sort button becomes turns white after pressing it (only visible in dark mode)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>Card alignment inconsistency</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B26" s="2" t="inlineStr">
         <is>
           <t>Shaharyar Haider</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>One of the cards is center aligned and one is right aligned, 
 Where does this target and budget in Daily consumption vs target comes from?,
@@ -862,187 +912,187 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>Card alignment inconsistency</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Shaharyar Haider</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="2" t="inlineStr">
         <is>
           <t>Exception not posting in the center of the card</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Card alignment inconsistency</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>One card is centered but the other is left aligned</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Graph missing connections / broken</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>broken chart and data isnt properly traversed(net usage is not divided rather reflected on everylevel)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Graph missing connections / broken</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Water graph has missing connections</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>Graph missing connections / broken</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
         <is>
           <t>CO2 graph has missing connections</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Graph missing connections / broken</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C32" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Energy Breakdown for water is not connected for Marina</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>Font/heading style inconsistency</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Chart Header, Pleacemnet of chart headers and Font Styles consistency is missing</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="2" t="inlineStr">
         <is>
           <t>Font/heading style inconsistency</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Font inconsistency</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Font/heading style inconsistency</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Title card font, alignment, and size is inconsistent</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="2" t="inlineStr">
         <is>
           <t>Font/heading style inconsistency</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Siji Wilson</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>AI Report - Temperature Statistics card Text alignment is not correct</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>No spaces in time labels (e.g., 6amTo6pm)</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B37" s="3" t="inlineStr">
         <is>
           <t>Shaharyar Haider</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C37" s="3" t="inlineStr">
         <is>
           <t>In "month" option this month graph is not showing at all
 also "PreviousWeek", "CurrentWeek", "PreviousMonth", "CurrentMonth" as no spaces in between the words</t>
@@ -1050,187 +1100,187 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>No spaces in time labels (e.g., 6amTo6pm)</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Site, Light - No spaces used in “6amTo6pm” and“6pmTo6am”</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="3" t="inlineStr">
         <is>
           <t>No spaces in time labels (e.g., 6amTo6pm)</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
         <is>
           <t>Site, Presence - No spaces used in “6amTo6pm” and“6pmTo6am”</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>No spaces in time labels (e.g., 6amTo6pm)</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Afrin Fathima</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>change card name daily Active hours (6am to 6pm) - Business Hours and afterhours</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>Legend / color coding issues</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>The color coding should be better for the numbers and should be distinguished from Alarm Severity or Device type.I had to pay attention to know that the alarms at number 2 and 4 are not "warnings" but "high" criticality alarms. The text of severity should be made a bit bigger or prominent. Because the number 2 is appearing yellow and my brain will be assosiating it with a warning instead of reading the fine print on the far right side about the actual severity</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>Legend / color coding issues</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Legend text is not shown completely</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>Legend / color coding issues</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>Shaharyar Haider</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Difficult to differentiate the Red color for HVAC and yellow combined with purple colour for overlapping Lights and Presence</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>Legend / color coding issues</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>No legend for colours?</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>Legend / color coding issues</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>There should be information, or legend on what the values mean for the values within the " ( ) ", and "3"</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="2" t="inlineStr">
         <is>
           <t>Legend / color coding issues</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="2" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>Full name of category is not displayed</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>Legend / color coding issues</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Current status Font color should match based on the legend given</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Legend / color coding issues</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Nihal Mascarenhas</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>color code not matching the pop window color code
 Dangerous color code is the color code for severe</t>
@@ -1238,68 +1288,68 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="3" t="inlineStr">
         <is>
           <t>Energy breakdown graph issues</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t>Shaharyar Haider</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="3" t="inlineStr">
         <is>
           <t>Visual missalignment in the Energy breakdown graph</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="3" t="inlineStr">
         <is>
           <t>Energy breakdown graph issues</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
         <is>
           <t>broken chart and data isnt properly traversed(net usage is not divided rather reflected on everylevel)</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="3" t="inlineStr">
         <is>
           <t>Energy breakdown graph issues</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>Energy Breakdown graph text is too small</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="3" t="inlineStr">
         <is>
           <t>Energy breakdown graph issues</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>Nihal Mascarenhas</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>1. Overlapping of waves
 2. Discontinuity of waves
@@ -1308,136 +1358,136 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>Alarm assignment shows null</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>While assigned the user email, It shows null null.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>Alarm assignment shows null</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Shaharyar Haider</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>under assignment of alarms vvengadesh circle is not showing with initials</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>Alarm assignment shows null</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Assigning alarms to people with no surname shows last name as null</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Roles not loading</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>While adding New Role, Role names are not shown. It's showing only "Loading Roles..."</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Roles not loading</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Roles never load</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>Units not specified</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Units are not present in "Total Estimated Annual Savings" under "AI Reports"</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>Units not specified</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Unit of Temperature should be specified</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="3" t="inlineStr">
         <is>
           <t>Full label/category text not displayed</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B60" s="3" t="inlineStr">
         <is>
           <t>Person 1</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="3" t="inlineStr">
         <is>
           <t>There is no way to read the full label text for tems in "Savings Potential by Category" under "AI Reports".
 Either the text should be scrolling or the widget should use the space on the right side</t>
@@ -1445,210 +1495,211 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>Full label/category text not displayed</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>Legend text is not shown completely</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="3" t="inlineStr">
         <is>
           <t>Full label/category text not displayed</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>Full name of category is not displayed</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="2" t="inlineStr">
         <is>
           <t>Heading size inconsistency in Settings/pages</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B63" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="2" t="inlineStr">
         <is>
           <t>In Settings Menu --&gt; Permission Matrix Heading is too big compare to other sub menus in settings</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>Heading size inconsistency in Settings/pages</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>In Settings Menu --&gt; Workflow Management Heading is too big compare to other sub menus in settings</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="2" t="inlineStr">
         <is>
           <t>Heading size inconsistency in Settings/pages</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
         <is>
           <t>Title card font, alignment, and size is inconsistent</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="2" t="inlineStr">
         <is>
           <t>Heading size inconsistency in Settings/pages</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="2" t="inlineStr">
         <is>
           <t>Siji Wilson</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C66" s="2" t="inlineStr">
         <is>
           <t>AI Report - Temperature Statistics card Text alignment is not correct</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="3" t="inlineStr">
         <is>
           <t>Issues and Recommendations card spacing/separation</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Ananth</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>Ananth</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>Issues and Recommendations should be separated in some way</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="3" t="inlineStr">
         <is>
           <t>Issues and Recommendations card spacing/separation</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>Siji Wilson</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>Space after Issues and recommendation card</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr">
         <is>
           <t>History / time window not working properly</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
+      <c r="B69" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C69" t="inlineStr">
+      <c r="C69" s="2" t="inlineStr">
         <is>
           <t>In Timewindow, History Tab, Grouping Interval selection is not updating.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>History / time window not working properly</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
+      <c r="B70" s="2" t="inlineStr">
         <is>
           <t>Vigneshwaran V</t>
         </is>
       </c>
-      <c r="C70" t="inlineStr">
+      <c r="C70" s="2" t="inlineStr">
         <is>
           <t>In Timewindow, If we update the time using Realtime tab It's updating correctly in the Last updated column based on selection. But, while updating using History it shows '1 second' as last updated time.</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>History / time window not working properly</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>Shaharyar Haider</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>History of data is not working, custom button is also not working</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="2" t="inlineStr">
         <is>
           <t>History / time window not working properly</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B72" s="2" t="inlineStr">
         <is>
           <t>Jezreel Phillip Alvarez</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C72" s="2" t="inlineStr">
         <is>
           <t>When custom is selected for Grouping interval for time window aggregation the days, minutes, seconds cannot be selected.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C72"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>